<commit_message>
updated chapter 4 code.
</commit_message>
<xml_diff>
--- a/stat4110-schedule.xlsx
+++ b/stat4110-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AliPe\Documents\GitHub Repositories\Ali-Raisolsadat.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B0D8D3-D2D7-4142-8DCB-75A454E1154D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32A100B-3D0C-4ED4-9D51-915CA49DD008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E80023EF-6428-48D2-ABA1-FC32C6C952F1}"/>
+    <workbookView xWindow="2730" yWindow="675" windowWidth="16995" windowHeight="14805" xr2:uid="{E80023EF-6428-48D2-ABA1-FC32C6C952F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
   <si>
     <t>Week (Mon–Fri)</t>
   </si>
@@ -167,9 +167,6 @@
     <t>Apr 13–17</t>
   </si>
   <si>
-    <t>Lecture 3 (Chapter 5)</t>
-  </si>
-  <si>
     <t>Deliverables</t>
   </si>
   <si>
@@ -213,6 +210,12 @@
   </si>
   <si>
     <t>Homework Review Chapter 3 &amp; Assignment 2 Review</t>
+  </si>
+  <si>
+    <t>Holiday (Easter)</t>
+  </si>
+  <si>
+    <t>Holiday (Good Friday)</t>
   </si>
 </sst>
 </file>
@@ -256,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -268,6 +271,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -628,7 +634,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -636,7 +642,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>20</v>
@@ -676,7 +682,7 @@
         <v>24</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>19</v>
@@ -696,7 +702,7 @@
         <v>25</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -730,7 +736,7 @@
         <v>11</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -744,7 +750,7 @@
         <v>41</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>19</v>
@@ -764,7 +770,7 @@
         <v>36</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -792,13 +798,13 @@
         <v>28</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -815,7 +821,7 @@
         <v>30</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -825,11 +831,11 @@
       <c r="B13" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>55</v>
+      <c r="C13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>59</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>19</v>
@@ -839,14 +845,14 @@
       <c r="A14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>51</v>
+      <c r="B14" s="5" t="s">
+        <v>58</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>19</v>
@@ -857,16 +863,16 @@
         <v>42</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>19</v>
+        <v>55</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>55</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>